<commit_message>
aCTUALIZACION CON CAMPOS NC-OE-PV-PP
</commit_message>
<xml_diff>
--- a/excel/1F.xlsx
+++ b/excel/1F.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dennis Ponce\Desktop\VISOR DE PROYECTOS EXCEL\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dennis Ponce\Desktop\sistema_de_control_de_cosechas\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8485F612-6C3D-42A8-BBC4-E770625D9CC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6711D59-4132-49FD-9C84-34954979279D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1050" yWindow="740" windowWidth="18150" windowHeight="9570" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="16">
   <si>
     <t>CICLO</t>
   </si>
@@ -61,6 +61,18 @@
   </si>
   <si>
     <t>CODIGO</t>
+  </si>
+  <si>
+    <t>NC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PV </t>
+  </si>
+  <si>
+    <t>PP</t>
   </si>
 </sst>
 </file>
@@ -134,11 +146,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -159,6 +168,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -449,178 +467,186 @@
     <col min="3" max="3" width="19.08984375" customWidth="1"/>
     <col min="4" max="4" width="15.81640625" customWidth="1"/>
     <col min="5" max="5" width="19.1796875" customWidth="1"/>
-    <col min="6" max="9" width="12.6328125" style="2" customWidth="1"/>
+    <col min="6" max="9" width="12.6328125" style="1" customWidth="1"/>
     <col min="10" max="13" width="12.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
+      <c r="J1" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="M1" s="9" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="6">
+      <c r="A2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5">
         <v>1198</v>
       </c>
-      <c r="C2" s="7">
-        <v>1</v>
-      </c>
-      <c r="D2" s="6">
+      <c r="C2" s="6">
+        <v>1</v>
+      </c>
+      <c r="D2" s="5">
         <v>16</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="5">
         <v>15</v>
       </c>
-      <c r="F2" s="8">
+      <c r="F2" s="7">
         <v>46219</v>
       </c>
-      <c r="G2" s="8">
+      <c r="G2" s="7">
         <v>46234</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="9">
-        <v>1</v>
-      </c>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
+      <c r="I2" s="8">
+        <v>1</v>
+      </c>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="6">
+      <c r="A3" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5">
         <v>1198</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="6">
         <v>6</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="5">
         <v>22</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="5">
         <v>15</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="7">
         <v>46195</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="7">
         <v>46208</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="9">
-        <v>1</v>
-      </c>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
+      <c r="I3" s="8">
+        <v>1</v>
+      </c>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="6">
+      <c r="A4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="5">
         <v>1198</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="6">
         <v>15</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <v>2</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>15</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="7">
         <v>46205</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="7">
         <v>46217</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="I4" s="9">
-        <v>1</v>
-      </c>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
+      <c r="I4" s="8">
+        <v>1</v>
+      </c>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="6">
+      <c r="A5" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5">
         <v>1198</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="6">
         <v>21</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="5">
         <v>7</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="5">
         <v>15</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="7">
         <v>46210</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="7">
         <v>46223</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="9">
-        <v>1</v>
-      </c>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
+      <c r="I5" s="8">
+        <v>1</v>
+      </c>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="B6" s="3"/>
-      <c r="G6" s="1"/>
+      <c r="B6" s="2"/>
+      <c r="G6" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>